<commit_message>
make Admin module in BMS project
</commit_message>
<xml_diff>
--- a/Backend/bloodmanagementproject/downloads/Users.xlsx
+++ b/Backend/bloodmanagementproject/downloads/Users.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="54">
   <si>
     <t>ID</t>
   </si>
@@ -35,31 +35,46 @@
     <t>STATUS</t>
   </si>
   <si>
-    <t>parth</t>
+    <t>Kevin</t>
+  </si>
+  <si>
+    <t>kevin@gmail.com</t>
+  </si>
+  <si>
+    <t>$2a$10$L.xpoWm4oTbH3dXUVP7Y6e1FiMQgPo1UH4z3sNQNJKv46KmCIRhsq</t>
+  </si>
+  <si>
+    <t>ADMIN</t>
+  </si>
+  <si>
+    <t>1234567890</t>
+  </si>
+  <si>
+    <t>ACTIVE</t>
+  </si>
+  <si>
+    <t>Parth</t>
   </si>
   <si>
     <t>parth@gmail.com</t>
   </si>
   <si>
-    <t>$2a$10$PSVtv7tSYkOSrWjMiL8bwOnwtu7FBAkt9dbN6sEwGVI3lhmmaOVnm</t>
+    <t>$2a$10$26JiqbCYtd8PLtRBckuQYuyLsVJ5cFb51TPzrCJ3GGQTslNO6jJg6</t>
   </si>
   <si>
     <t>DONOR</t>
   </si>
   <si>
-    <t>9876543210</t>
-  </si>
-  <si>
-    <t>ACTIVE</t>
-  </si>
-  <si>
-    <t>Kevin</t>
-  </si>
-  <si>
-    <t>kevin@gmail.com</t>
-  </si>
-  <si>
-    <t>$2a$10$2epS0O4yX0r.JLT7.J0rM.wbIm6gKB7T4FUHZj7P.Z64oon5StqM6</t>
+    <t>Dinesh</t>
+  </si>
+  <si>
+    <t>dinesh@gmail.com</t>
+  </si>
+  <si>
+    <t>$2a$10$5xyw6GR1d088yj/s60dYce4Nhx41//m5ggZGadQBwRdB5FRxxDsaS</t>
+  </si>
+  <si>
+    <t>USER</t>
   </si>
   <si>
     <t>Aditya</t>
@@ -68,19 +83,10 @@
     <t>adi@gmail.com</t>
   </si>
   <si>
-    <t>$2a$10$yUZT5qHULoKk1O9cV4Gub.IgRHWmMyDg7s3tiGBvJ2nmas4YJ.Pg.</t>
-  </si>
-  <si>
-    <t>USER</t>
-  </si>
-  <si>
-    <t>Dinesh</t>
-  </si>
-  <si>
-    <t>dinesh@gmail.com</t>
-  </si>
-  <si>
-    <t>$2a$10$/uh8bklSZY.gAeL6Ca3zq.zk75/35eDZ6B8aowtO0AN3JD5mEj86u</t>
+    <t>$2a$10$BePieWk52tmrfJ6hufi.MO9sAJ.ZYpI/tHjR.0.3WAiDdD5nqOCMi</t>
+  </si>
+  <si>
+    <t>HOSPITAL</t>
   </si>
   <si>
     <t>Smit</t>
@@ -89,10 +95,73 @@
     <t>smit@gmail.com</t>
   </si>
   <si>
-    <t>$2a$10$7rZZXTzY4VwJWgrnI5feuOs7TZ4DmGCj1QIUR.5G73uCNzTTErc2e</t>
-  </si>
-  <si>
-    <t>HOSPITAL</t>
+    <t>$2a$10$TG7fRy73ujRZbOvcIqrxLunpReQcdNCPTXsGOvScoTunNNmlWHyeq</t>
+  </si>
+  <si>
+    <t>Dev</t>
+  </si>
+  <si>
+    <t>dev@gmail.com</t>
+  </si>
+  <si>
+    <t>$2a$10$5n14jD8NOG219WGRNUe7AuJtkQW5TnaXgwPjqMVku5RHLqnOa0Lza</t>
+  </si>
+  <si>
+    <t>hani</t>
+  </si>
+  <si>
+    <t>hani@gmail.com</t>
+  </si>
+  <si>
+    <t>$2a$10$oN3RxjYw8ZbzcS7DthM2u.h6PoxaRexZAga/1QyvQRHLCsTDScpu.</t>
+  </si>
+  <si>
+    <t>5465324544</t>
+  </si>
+  <si>
+    <t>INACTIVE</t>
+  </si>
+  <si>
+    <t>miten</t>
+  </si>
+  <si>
+    <t>miten@gmail.com</t>
+  </si>
+  <si>
+    <t>$2a$10$uTqRiqPkjhgMxUXxjnrbO.FiE8Px23qanQKjKoMjIRhgYkEZu6NKa</t>
+  </si>
+  <si>
+    <t>jay</t>
+  </si>
+  <si>
+    <t>jay@gmail.com</t>
+  </si>
+  <si>
+    <t>$2a$10$p5WUFsghBsaPIvipvFmA5.lkZwghQqKlHXSjtPS9ZbcAU0ePF0bRm</t>
+  </si>
+  <si>
+    <t>fenny</t>
+  </si>
+  <si>
+    <t>fenny@gmail.com</t>
+  </si>
+  <si>
+    <t>$2a$10$l1HsPqN62Wis1H8GFAfir.qijtACwOHv.XIp78PdGE4cTvJ1uJWP.</t>
+  </si>
+  <si>
+    <t>7854123698</t>
+  </si>
+  <si>
+    <t>Maharshi</t>
+  </si>
+  <si>
+    <t>maharshi@gmail.com</t>
+  </si>
+  <si>
+    <t>$2a$10$0pWRuuRa7H3VvCEn0E/01ebNBzIq9N/5zRWdph6jV3C8ZNKC2x0Ee</t>
+  </si>
+  <si>
+    <t>8754215874</t>
   </si>
   <si>
     <t>Divyang</t>
@@ -101,31 +170,10 @@
     <t>divyang@gmail.com</t>
   </si>
   <si>
-    <t>$2a$10$ev3mTJtGnLItWOrw8spVp.tXLHbiThjlRoK8Gp9UD8ZPRZ1T.MIJu</t>
-  </si>
-  <si>
-    <t>ADMIN</t>
-  </si>
-  <si>
-    <t>Chirag</t>
-  </si>
-  <si>
-    <t>chch@gmail.com</t>
-  </si>
-  <si>
-    <t>$2a$10$lyJFdXIEkLU4nG/wM.ybs.5XzWOVLOVlN.J8YFdSzYFr9JJLXPSBq</t>
-  </si>
-  <si>
-    <t>Ravi</t>
-  </si>
-  <si>
-    <t>ravi@gmail.com</t>
-  </si>
-  <si>
-    <t>$2a$10$iinlJmMv2043f1U6aTUZ.uKVe/T9YGbvBIPR5FSI2vpM.ylaJDFqa</t>
-  </si>
-  <si>
-    <t>1234567890</t>
+    <t>$2a$10$fnw6SjKzUv2Ey7ZA2LYTjuj65LR0.g.RyFX.a6yzjPwoSJAak8RhW</t>
+  </si>
+  <si>
+    <t>9965875463</t>
   </si>
 </sst>
 </file>
@@ -170,7 +218,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -233,7 +281,7 @@
         <v>15</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F3" t="s" s="0">
         <v>11</v>
@@ -244,19 +292,19 @@
     </row>
     <row r="4">
       <c r="A4" t="n" s="0">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F4" t="s" s="0">
         <v>11</v>
@@ -267,19 +315,19 @@
     </row>
     <row r="5">
       <c r="A5" t="n" s="0">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F5" t="s" s="0">
         <v>11</v>
@@ -290,19 +338,19 @@
     </row>
     <row r="6">
       <c r="A6" t="n" s="0">
-        <v>5.0</v>
+        <v>6.0</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C6" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="E6" t="s" s="0">
         <v>24</v>
-      </c>
-      <c r="D6" t="s" s="0">
-        <v>25</v>
-      </c>
-      <c r="E6" t="s" s="0">
-        <v>26</v>
       </c>
       <c r="F6" t="s" s="0">
         <v>11</v>
@@ -313,19 +361,19 @@
     </row>
     <row r="7">
       <c r="A7" t="n" s="0">
-        <v>6.0</v>
+        <v>8.0</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F7" t="s" s="0">
         <v>11</v>
@@ -336,7 +384,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n" s="0">
-        <v>7.0</v>
+        <v>9.0</v>
       </c>
       <c r="B8" t="s" s="0">
         <v>31</v>
@@ -348,35 +396,127 @@
         <v>33</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F8" t="s" s="0">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="G8" t="s" s="0">
-        <v>12</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n" s="0">
-        <v>8.0</v>
+        <v>10.0</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C9" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="F9" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="G9" t="s" s="0">
         <v>35</v>
       </c>
-      <c r="D9" t="s" s="0">
-        <v>36</v>
-      </c>
-      <c r="E9" t="s" s="0">
+    </row>
+    <row r="10">
+      <c r="A10" t="n" s="0">
+        <v>13.0</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="F10" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="G10" t="s" s="0">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n" s="0">
+        <v>19.0</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="E11" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="F11" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="G11" t="s" s="0">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n" s="0">
+        <v>20.0</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>47</v>
+      </c>
+      <c r="D12" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="E12" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="F12" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="G12" t="s" s="0">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n" s="0">
+        <v>21.0</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>51</v>
+      </c>
+      <c r="D13" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="E13" t="s" s="0">
         <v>10</v>
       </c>
-      <c r="F9" t="s" s="0">
-        <v>37</v>
-      </c>
-      <c r="G9" t="s" s="0">
+      <c r="F13" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="G13" t="s" s="0">
         <v>12</v>
       </c>
     </row>

</xml_diff>